<commit_message>
Add internal-only combined cash position sheet to the structuring analysis
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tace5U23AKexiDyfCZxMPM
</commit_message>
<xml_diff>
--- a/output/01_Structuring_Analysis.xlsx
+++ b/output/01_Structuring_Analysis.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OptB_Cash" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage_S1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions_Log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined_Position" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4342,4 +4343,669 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INTERNAL ONLY: combined Green Square + L'avenir cash position (Jalour level). Never include in any investor pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cumulative net cash flow before any investor instrument, EGP million, base case, from the edited source model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Green Square cumulative</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>L'avenir cumulative</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Combined cumulative</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>-91.25</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>-91.25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>-102.5</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>-102.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>-98.61076249999999</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>-98.61076249999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>-79.58228749999999</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>-85</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>-164.5822875</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>-78.57028124999999</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>-89.38435</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-167.95463125</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>-68.68474375</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>-75.65304999999999</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>-144.33779375</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>-86.93043374999999</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>-62.892225</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>-149.82265875</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>-88.42826437499998</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>-46.733835</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>-135.162099375</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>-81.73067593749997</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>-85.13881000000001</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>-166.8694859375</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>339.8919015625002</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>-102.0180625</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>237.8738390625002</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>478.6586415625002</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>-100.9419475</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>377.7166940625002</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>608.3816315625002</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>-77.89594749999998</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>530.4856840625002</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>514.9943415625002</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>-32.89763124999998</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>482.0967103125002</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>394.0435103125001</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>22.28235125</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>416.3258615625001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>222.4926790625001</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>503.5783587499998</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>726.0710378125</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>104.3235146875001</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>473.4240912499998</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>577.7476059374999</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>120.5501543750001</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>344.1903637499997</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>464.7405181249999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>135.2628703125001</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>245.7470362499997</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>381.0099065624998</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>143.9868150000001</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>282.5470237499997</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>426.5338387499997</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>148.3697596875001</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>317.5354462499996</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>465.9052059374997</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>175.2527043750001</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>372.3149081249996</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>547.5676124999998</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>194.8554303125001</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>419.9683218749996</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>614.8237521874997</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>214.4581562500001</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>458.8061981249996</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>673.2643543749997</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>234.0608821875001</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>487.3524468749995</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>721.4133290624997</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>270.3756081250001</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>538.3986956249995</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>808.7743037499996</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>303.4142356250001</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>589.4449443749995</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>892.8591799999997</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>332.8444068750001</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>640.4911931249995</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>973.3355999999997</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>357.9335781250001</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>691.5374418749996</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>1049.47102</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>275.2645390234376</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>494.2772134374998</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>769.5417524609373</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>289.3771978515626</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>514.9865045312497</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>804.3637023828123</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>303.4898566796876</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>533.5256917187496</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>837.0155483984372</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>317.6025155078126</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>549.8947749999996</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>867.4972905078123</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>331.7151743359376</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>562.7665314062497</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>894.4817057421873</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>344.5992962500001</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>573.6128574999997</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>918.2121537499997</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>105</v>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>357.4834181640626</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>583.0648656249997</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>940.5482837890623</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>108</v>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>368.0244175000001</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>587.1408868749996</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>955.1653043749998</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>111</v>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>373.4391367187501</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>591.2169081249996</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>964.6560448437497</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>375.4475275000001</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>595.2929293749995</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>970.7404568749996</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>117</v>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>375.4475275000001</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>595.2929293749995</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>970.7404568749996</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>375.4475275000001</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>595.2929293749995</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>970.7404568749996</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>123</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>375.4475275000001</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>595.2929293749995</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>970.7404568749996</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>375.4475275000001</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>595.2929293749995</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>970.7404568749996</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>129</v>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>375.4475275000001</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>595.2929293749995</v>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>970.7404568749996</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Lowest combined position: -168.0 at month 15 (Green Square alone -102.5; L'avenir alone -102.0).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild all packs on the standalone project models (own timelines), remove retained-unit wording, add source models
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tace5U23AKexiDyfCZxMPM
</commit_message>
<xml_diff>
--- a/output/01_Structuring_Analysis.xlsx
+++ b/output/01_Structuring_Analysis.xlsx
@@ -485,14 +485,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source of truth: ALAHLY-SABBOUR MOSTAKBAL CITY -V2.xlsx. Results computed in Python (_build/engine2.py, packdata.py); the Financial Annexes recompute them with live formulas and tie to these values.</t>
+          <t>Source of truth: the two standalone project models (Green_Square.xlsx, Lavenir.xlsx; each project month 1 is its own sales launch). Results computed in Python (_build/engine2.py, packdata.py); the Financial Annexes recompute them with live formulas and tie to these values.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>EGP million unless stated. NPV and IRR on quarter-end months, discount rate 14% (kept by Jalour). Investor funds at GS month 3 / LA month 12.</t>
+          <t>EGP million unless stated. NPV and IRR on quarter-end months, discount rate 14% (kept by Jalour). Investor funds at GS month -3 / LA month 0 (each project own timeline; combined view uses a common calendar with GS launch = month 1 and L'avenir launch = month 7).</t>
         </is>
       </c>
     </row>
@@ -788,13 +788,13 @@
         <v>375.4475275000002</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>215.311392548924</v>
+        <v>229.8896586798693</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>-102.5</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -812,13 +812,13 @@
         <v>257.72937475</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>-33.59468460746148</v>
+        <v>-35.86930764061781</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>-441.19460834375</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -836,13 +836,13 @@
         <v>493.1656802500001</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>314.5815929584118</v>
+        <v>335.8812284665625</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>-102.5</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -860,13 +860,13 @@
         <v>295.2741275000001</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>162.3456810366187</v>
+        <v>173.3377540307293</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>-102.5</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -884,13 +884,13 @@
         <v>375.4475275000001</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>125.4642192885034</v>
+        <v>133.9591287173367</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>-235.690784375</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -908,13 +908,13 @@
         <v>375.4475275</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>155.3293249012312</v>
+        <v>165.8463356805642</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>-269.1979209375</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
@@ -932,13 +932,13 @@
         <v>257.7293747499999</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>-80.94894853985042</v>
+        <v>-86.42982579796387</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>-729.38647159375</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
@@ -956,13 +956,13 @@
         <v>595.2929293749995</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>307.5323710915292</v>
+        <v>350.5869030443433</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>-102.0180625</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -980,13 +980,13 @@
         <v>455.5902364374995</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>39.8977448934632</v>
+        <v>45.48342917854805</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>-848.6042838750002</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
@@ -1004,13 +1004,13 @@
         <v>734.9956223124996</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>411.5481560868075</v>
+        <v>469.1648979389606</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>-87.572785</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1028,13 +1028,13 @@
         <v>515.1195293749996</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>257.9254371887749</v>
+        <v>294.0349983952034</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>-116.9499475</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -1052,13 +1052,13 @@
         <v>595.2929293749996</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>209.2786594690933</v>
+        <v>238.5776717947664</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>-381.30656875</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
@@ -1076,13 +1076,13 @@
         <v>595.2929293749996</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>274.5391799076958</v>
+        <v>312.9746650947733</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>-244.3073362500001</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
@@ -1100,13 +1100,13 @@
         <v>455.5902364374997</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>13.85048869570005</v>
+        <v>15.78955711309806</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>-848.6042838750002</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1804,7 +1804,7 @@
         <v>0.2074195733610894</v>
       </c>
       <c r="R5" s="5" t="n">
-        <v>-9.546510458546674</v>
+        <v>-10.19288391997381</v>
       </c>
       <c r="S5" s="5" t="n">
         <v>-46</v>
@@ -1816,7 +1816,7 @@
         <v>0.3071735011044534</v>
       </c>
       <c r="V5" s="5" t="n">
-        <v>-23.89878315078667</v>
+        <v>-25.51691778292767</v>
       </c>
     </row>
     <row r="6">
@@ -1874,7 +1874,7 @@
         <v>0.2074195733610893</v>
       </c>
       <c r="R6" s="5" t="n">
-        <v>-14.31976568782</v>
+        <v>-15.28932587996071</v>
       </c>
       <c r="S6" s="5" t="n">
         <v>-69</v>
@@ -1886,7 +1886,7 @@
         <v>0.3071735011044534</v>
       </c>
       <c r="V6" s="5" t="n">
-        <v>-35.84817472618001</v>
+        <v>-38.2753766743915</v>
       </c>
     </row>
     <row r="7">
@@ -1944,7 +1944,7 @@
         <v>0.2074195733610894</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>-19.09302091709335</v>
+        <v>-20.38576783994763</v>
       </c>
       <c r="S7" s="5" t="n">
         <v>-92</v>
@@ -1956,7 +1956,7 @@
         <v>0.3071735011044534</v>
       </c>
       <c r="V7" s="5" t="n">
-        <v>-47.79756630157333</v>
+        <v>-51.03383556585533</v>
       </c>
     </row>
     <row r="8">
@@ -2014,7 +2014,7 @@
         <v>0.2074195733610893</v>
       </c>
       <c r="R8" s="5" t="n">
-        <v>-23.86627614636671</v>
+        <v>-25.48220979993456</v>
       </c>
       <c r="S8" s="5" t="n">
         <v>-115</v>
@@ -2026,7 +2026,7 @@
         <v>0.3071735011044535</v>
       </c>
       <c r="V8" s="5" t="n">
-        <v>-59.7469578769667</v>
+        <v>-63.79229445731919</v>
       </c>
     </row>
     <row r="9">
@@ -2084,7 +2084,7 @@
         <v>0.225573897725654</v>
       </c>
       <c r="R9" s="5" t="n">
-        <v>-10.40125533765831</v>
+        <v>-11.85743108493047</v>
       </c>
       <c r="S9" s="5" t="n">
         <v>-46</v>
@@ -2096,7 +2096,7 @@
         <v>0.3158693984401545</v>
       </c>
       <c r="V9" s="5" t="n">
-        <v>-22.4651194246602</v>
+        <v>-25.61023614411263</v>
       </c>
     </row>
     <row r="10">
@@ -2154,7 +2154,7 @@
         <v>0.2255738977256541</v>
       </c>
       <c r="R10" s="5" t="n">
-        <v>-15.60188300648746</v>
+        <v>-17.78614662739571</v>
       </c>
       <c r="S10" s="5" t="n">
         <v>-69.00000000000001</v>
@@ -2166,7 +2166,7 @@
         <v>0.3158693984401545</v>
       </c>
       <c r="V10" s="5" t="n">
-        <v>-33.6976791369903</v>
+        <v>-38.41535421616895</v>
       </c>
     </row>
     <row r="11">
@@ -2224,7 +2224,7 @@
         <v>0.225573897725654</v>
       </c>
       <c r="R11" s="5" t="n">
-        <v>-20.80251067531661</v>
+        <v>-23.71486216986094</v>
       </c>
       <c r="S11" s="5" t="n">
         <v>-92</v>
@@ -2236,7 +2236,7 @@
         <v>0.3158693984401545</v>
       </c>
       <c r="V11" s="5" t="n">
-        <v>-44.9302388493204</v>
+        <v>-51.22047228822527</v>
       </c>
     </row>
     <row r="12">
@@ -2294,7 +2294,7 @@
         <v>0.225573897725654</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>-26.00313834414577</v>
+        <v>-29.64357771232618</v>
       </c>
       <c r="S12" s="5" t="n">
         <v>-115</v>
@@ -2306,7 +2306,7 @@
         <v>0.3158693984401545</v>
       </c>
       <c r="V12" s="5" t="n">
-        <v>-56.16279856165052</v>
+        <v>-64.0255903602816</v>
       </c>
     </row>
   </sheetData>
@@ -2455,7 +2455,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>-21.26828942239149</v>
+        <v>-22.70831904497237</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>-17.90095630434783</v>
@@ -2481,7 +2481,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -2508,7 +2508,7 @@
         <v>0.2902766281599988</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>-23.73837492533987</v>
+        <v>-25.34564866539117</v>
       </c>
       <c r="H6" s="10" t="n">
         <v>-19.45975868259913</v>
@@ -2534,7 +2534,7 @@
         <v>0.2634662535782694</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
@@ -2561,7 +2561,7 @@
         <v>0.278352764925566</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>-22.55546338112543</v>
+        <v>-24.0826447531103</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>-19.6302963881863</v>
@@ -2587,7 +2587,7 @@
         <v>0.2613363690787225</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -2614,7 +2614,7 @@
         <v>0.2654639948399947</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-31.90243413358723</v>
+        <v>-34.06247856745856</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>-11.93397086956522</v>
@@ -2640,7 +2640,7 @@
         <v>0.2654639948399947</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
@@ -2667,7 +2667,7 @@
         <v>0.2902766284723172</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>-35.60756243723743</v>
+        <v>-38.01847305064749</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>-12.97317239490064</v>
@@ -2693,7 +2693,7 @@
         <v>0.2634662539104816</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
@@ -2720,7 +2720,7 @@
         <v>0.2783527649255662</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-33.83319507168816</v>
+        <v>-36.12396712966546</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>-13.08686425879087</v>
@@ -2746,7 +2746,7 @@
         <v>0.2613363690787225</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11">
@@ -2773,7 +2773,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>-42.53657884478297</v>
+        <v>-45.41663808994474</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>-8.950478152173913</v>
@@ -2799,7 +2799,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12">
@@ -2826,7 +2826,7 @@
         <v>0.2902766286284764</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-47.47674994913497</v>
+        <v>-50.69129743590376</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>-9.729879273613443</v>
@@ -2852,7 +2852,7 @@
         <v>0.2634662540765875</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -2879,7 +2879,7 @@
         <v>0.278352764925566</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>-45.11092676225087</v>
+        <v>-48.1652895062206</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>-9.815148194093149</v>
@@ -2905,7 +2905,7 @@
         <v>0.2613363690787225</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14">
@@ -2932,7 +2932,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-53.1707235559787</v>
+        <v>-56.77079761243091</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>-7.16038252173913</v>
@@ -2958,7 +2958,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15">
@@ -2985,7 +2985,7 @@
         <v>0.2902766287221718</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-59.34593746103251</v>
+        <v>-63.36412182116005</v>
       </c>
       <c r="H15" s="10" t="n">
         <v>-7.783903408060977</v>
@@ -3011,7 +3011,7 @@
         <v>0.2634662541762513</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
@@ -3038,7 +3038,7 @@
         <v>0.2783527649255661</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-56.38865845281359</v>
+        <v>-60.20661188277575</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>-7.852118555274519</v>
@@ -3064,7 +3064,7 @@
         <v>0.2613363690787225</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17">
@@ -3091,7 +3091,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>-19.27764254549257</v>
+        <v>-21.97651250186154</v>
       </c>
       <c r="H17" s="10" t="n">
         <v>-13.48525852173914</v>
@@ -3117,7 +3117,7 @@
         <v>0.2654639948399945</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18">
@@ -3144,7 +3144,7 @@
         <v>0.2865766172362276</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-21.23451406294631</v>
+        <v>-24.2073460317588</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>-11.64578820397757</v>
@@ -3170,7 +3170,7 @@
         <v>0.2575142685070789</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
@@ -3197,7 +3197,7 @@
         <v>0.273781615486074</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>-20.06803854543199</v>
+        <v>-22.87756394179247</v>
       </c>
       <c r="H19" s="10" t="n">
         <v>-14.15912392399709</v>
@@ -3223,7 +3223,7 @@
         <v>0.2586309861149937</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20">
@@ -3250,7 +3250,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>-28.91646381823889</v>
+        <v>-32.96476875279234</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>-8.990172347826093</v>
@@ -3276,7 +3276,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21">
@@ -3303,7 +3303,7 @@
         <v>0.2865766176394661</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-31.85177115100156</v>
+        <v>-36.31101911214178</v>
       </c>
       <c r="H21" s="10" t="n">
         <v>-7.763858772646461</v>
@@ -3329,7 +3329,7 @@
         <v>0.2575142688415505</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22">
@@ -3356,7 +3356,7 @@
         <v>0.2737816154860739</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-30.102057818148</v>
+        <v>-34.31634591268872</v>
       </c>
       <c r="H22" s="10" t="n">
         <v>-9.439415949331392</v>
@@ -3382,7 +3382,7 @@
         <v>0.2586309861149937</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23">
@@ -3409,7 +3409,7 @@
         <v>0.2654639948399946</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>-38.55528509098514</v>
+        <v>-43.95302500372307</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>-6.742629260869569</v>
@@ -3435,7 +3435,7 @@
         <v>0.2654639948399945</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24">
@@ -3462,7 +3462,7 @@
         <v>0.2865766178410853</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>-42.46902823905678</v>
+        <v>-48.41469219252473</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>-5.822894068232876</v>
@@ -3488,7 +3488,7 @@
         <v>0.2575142690087864</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25">
@@ -3515,7 +3515,7 @@
         <v>0.273781615486074</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>-40.13607709086398</v>
+        <v>-45.75512788358494</v>
       </c>
       <c r="H25" s="10" t="n">
         <v>-7.079561961998546</v>
@@ -3541,7 +3541,7 @@
         <v>0.2586309861149937</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26">
@@ -3568,7 +3568,7 @@
         <v>0.2654639948399944</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>-48.19410636373144</v>
+        <v>-54.94128125465385</v>
       </c>
       <c r="H26" s="10" t="n">
         <v>-5.394103408695655</v>
@@ -3594,7 +3594,7 @@
         <v>0.2654639948399945</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27">
@@ -3621,7 +3621,7 @@
         <v>0.2865766179620571</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>-53.08628532711207</v>
+        <v>-60.51836527290777</v>
       </c>
       <c r="H27" s="10" t="n">
         <v>-4.658315249185357</v>
@@ -3647,7 +3647,7 @@
         <v>0.2575142691091277</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28">
@@ -3674,7 +3674,7 @@
         <v>0.273781615486074</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>-50.17009636358</v>
+        <v>-57.19390985448121</v>
       </c>
       <c r="H28" s="10" t="n">
         <v>-5.663649569598835</v>
@@ -3700,7 +3700,7 @@
         <v>0.2586309861149937</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -3767,7 +3767,7 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>421.6225775000001</v>
@@ -3784,7 +3784,7 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>138.76674</v>
@@ -3801,7 +3801,7 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>129.72299</v>
@@ -3818,7 +3818,7 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>-93.38729000000001</v>
@@ -3835,7 +3835,7 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>-120.95083125</v>
@@ -3852,7 +3852,7 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>-171.55083125</v>
@@ -3869,7 +3869,7 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>-118.169164375</v>
@@ -3886,7 +3886,7 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>16.2266396875</v>
@@ -3903,7 +3903,7 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>14.7127159375</v>
@@ -3920,7 +3920,7 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>8.723944687500001</v>
@@ -3937,7 +3937,7 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>4.3829446875</v>
@@ -3954,7 +3954,7 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>26.8829446875</v>
@@ -4005,7 +4005,7 @@
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>44.99831625</v>
@@ -4022,7 +4022,7 @@
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>55.17998249999998</v>
@@ -4039,7 +4039,7 @@
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>481.2960074999998</v>
@@ -4056,7 +4056,7 @@
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B24" s="5" t="n">
         <v>-30.15426749999999</v>
@@ -4073,7 +4073,7 @@
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B25" s="5" t="n">
         <v>-129.2337275000001</v>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="B26" s="5" t="n">
         <v>-98.44332750000007</v>
@@ -4107,7 +4107,7 @@
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>36.79998749999996</v>
@@ -4124,7 +4124,7 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>34.98842249999996</v>
@@ -4141,7 +4141,7 @@
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B29" s="5" t="n">
         <v>54.779461875</v>
@@ -4158,7 +4158,7 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="B30" s="5" t="n">
         <v>47.65341375000001</v>
@@ -4175,7 +4175,7 @@
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="B31" s="5" t="n">
         <v>38.83787624999999</v>
@@ -4192,7 +4192,7 @@
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B32" s="5" t="n">
         <v>28.54624874999998</v>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Investor funds 100% at t0 (GS M3, LA M12); pooled with project cash, no restricted account.</t>
+          <t>Investor funds 100% at t0 (GS month -3, LA month 0); pooled with project cash, no restricted account.</t>
         </is>
       </c>
     </row>

</xml_diff>